<commit_message>
vengeanceaiUSC-LBOMODEL1: load ZoomInfo figures into LBO template
Replace BMC sample inputs with GTM/ZI public data (FY2025 P&L, Q2’26
debt/cash/shares, market price), rebuild Sources & Uses and forecast with
S&M efficiency path, and refresh sponsor MoIC/IRR summary.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LBO_Complex_Template_IRR_MoM.xlsx
+++ b/LBO_Complex_Template_IRR_MoM.xlsx
@@ -94,61 +94,61 @@
     <numFmt numFmtId="187" formatCode="0\A"/>
     <numFmt numFmtId="188" formatCode="General\ &quot;yrs&quot;"/>
     <numFmt numFmtId="189" formatCode="0.000%"/>
-    <numFmt numFmtId="190" formatCode="#,##0.00_);\(#,##0\)"/>
-    <numFmt numFmtId="191" formatCode="#,##0.0%_);\(#,##0.0%\)"/>
-    <numFmt numFmtId="192" formatCode="0.0\ \x"/>
-    <numFmt numFmtId="193" formatCode="#,##0.00\ ;\(#,##0.00\)"/>
-    <numFmt numFmtId="194" formatCode="&quot;$&quot;#,##0.00\ ;\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="195" formatCode="0.0%_);\(0.0%\)"/>
-    <numFmt numFmtId="196" formatCode="0.000\ \x&quot;rate&quot;"/>
-    <numFmt numFmtId="197" formatCode="#,##0.000_);[Red]\(#,##0.000\)"/>
-    <numFmt numFmtId="198" formatCode="0.00_);\(0.00\);0.00"/>
-    <numFmt numFmtId="199" formatCode="\C&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="200" formatCode="#,##0%_);\(#,##0.0%\)"/>
-    <numFmt numFmtId="201" formatCode="_(* #,##0.00000000_);_(* \(#,##0.00000000\);_(* &quot;-&quot;?_);_(@_)"/>
-    <numFmt numFmtId="202" formatCode="mmm\-d\-yyyy"/>
-    <numFmt numFmtId="203" formatCode="mmm\-yyyy"/>
-    <numFmt numFmtId="204" formatCode="yyyy"/>
-    <numFmt numFmtId="205" formatCode="0.00\x&quot;rate&quot;"/>
-    <numFmt numFmtId="206" formatCode="0.0&quot;  &quot;"/>
-    <numFmt numFmtId="207" formatCode="&quot;$&quot;#,##0.0\ ;[Red]\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="208" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;?_);_(@_)"/>
-    <numFmt numFmtId="209" formatCode="&quot;$&quot;#,##0.000_);[Red]\(&quot;$&quot;#,##0.000\)"/>
-    <numFmt numFmtId="210" formatCode="&quot;$&quot;#,##0.00&quot;A&quot;;[Red]\(&quot;$&quot;#,##0.00\)&quot;A&quot;"/>
-    <numFmt numFmtId="211" formatCode="#,##0.0\ ;[Red]\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="212" formatCode="&quot;$&quot;#,##0.00&quot;E&quot;;[Red]\(&quot;$&quot;#,##0.00\)&quot;E&quot;"/>
-    <numFmt numFmtId="213" formatCode="_([$€-2]* #,##0.00_);_([$€-2]* \(#,##0.00\);_([$€-2]* &quot;-&quot;??_)"/>
-    <numFmt numFmtId="214" formatCode="#,##0.00;\(#,##0.00\)"/>
-    <numFmt numFmtId="215" formatCode=".%\,\(0.0%%;\t"/>
-    <numFmt numFmtId="216" formatCode="#,##0.0_);[Red]\(#,##0.0\)"/>
-    <numFmt numFmtId="217" formatCode="0.0%_);[Red]\(0.0%\)"/>
-    <numFmt numFmtId="218" formatCode="0.00_);\(0.00\);0.00_)"/>
-    <numFmt numFmtId="219" formatCode="#,##0\x"/>
-    <numFmt numFmtId="220" formatCode="&quot;TKR&quot;\ 0"/>
-    <numFmt numFmtId="221" formatCode=".%\,\(0.%%;\t"/>
-    <numFmt numFmtId="222" formatCode="&quot;$&quot;#,###.0\ \ "/>
-    <numFmt numFmtId="223" formatCode="#,##0.00\x_);[Red]\(#,##0.00\x\)"/>
-    <numFmt numFmtId="224" formatCode="#,##0.000_);\(#,##0.000\)"/>
-    <numFmt numFmtId="225" formatCode="#,##0.00\x_);[Red]\(#,##0.00\x\);&quot;--  &quot;"/>
-    <numFmt numFmtId="226" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="227" formatCode="0.0\x_);[Red]\(0.0\x\)"/>
-    <numFmt numFmtId="228" formatCode="0.0\ "/>
-    <numFmt numFmtId="229" formatCode="&quot;$&quot;#,##0.0;\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="230" formatCode="#,##0.00%_);\(#,##0.00%\)"/>
-    <numFmt numFmtId="231" formatCode="0.00\%;\-0.00\%;0.00\%"/>
-    <numFmt numFmtId="232" formatCode="0.0%\ ;\(0.0%\)"/>
-    <numFmt numFmtId="233" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="234" formatCode="&quot;$&quot;0.00\ "/>
-    <numFmt numFmtId="235" formatCode="0.0\ \ \ \ \ "/>
-    <numFmt numFmtId="236" formatCode="0.00\x;\-0.00\x;0.00\x"/>
-    <numFmt numFmtId="237" formatCode="&quot;$&quot;#,##0.000_);\(&quot;$&quot;#,##0.000\)"/>
-    <numFmt numFmtId="238" formatCode="#,##0.0_);\(#,##0.0\);_(* &quot;-&quot;_)"/>
-    <numFmt numFmtId="239" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="240" formatCode="0.00%_);[Red]\(0.00%\)"/>
-    <numFmt numFmtId="241" formatCode="#,##0.0\x_);\(#,##0.0\x\)"/>
-    <numFmt numFmtId="242" formatCode="#,##0.00\x_);\(#,##0.00\x\)"/>
-    <numFmt numFmtId="243" formatCode="###0&quot;E&quot;_)"/>
-    <numFmt numFmtId="244" formatCode="#,##0.0"/>
+    <numFmt numFmtId="190" formatCode="#,##0.0"/>
+    <numFmt numFmtId="191" formatCode="#,##0.00_);\(#,##0\)"/>
+    <numFmt numFmtId="192" formatCode="#,##0.0%_);\(#,##0.0%\)"/>
+    <numFmt numFmtId="193" formatCode="0.0\ \x"/>
+    <numFmt numFmtId="194" formatCode="#,##0.00\ ;\(#,##0.00\)"/>
+    <numFmt numFmtId="195" formatCode="&quot;$&quot;#,##0.00\ ;\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="196" formatCode="0.0%_);\(0.0%\)"/>
+    <numFmt numFmtId="197" formatCode="0.000\ \x&quot;rate&quot;"/>
+    <numFmt numFmtId="198" formatCode="#,##0.000_);[Red]\(#,##0.000\)"/>
+    <numFmt numFmtId="199" formatCode="0.00_);\(0.00\);0.00"/>
+    <numFmt numFmtId="200" formatCode="\C&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="201" formatCode="#,##0%_);\(#,##0.0%\)"/>
+    <numFmt numFmtId="202" formatCode="_(* #,##0.00000000_);_(* \(#,##0.00000000\);_(* &quot;-&quot;?_);_(@_)"/>
+    <numFmt numFmtId="203" formatCode="mmm\-d\-yyyy"/>
+    <numFmt numFmtId="204" formatCode="mmm\-yyyy"/>
+    <numFmt numFmtId="205" formatCode="yyyy"/>
+    <numFmt numFmtId="206" formatCode="0.00\x&quot;rate&quot;"/>
+    <numFmt numFmtId="207" formatCode="0.0&quot;  &quot;"/>
+    <numFmt numFmtId="208" formatCode="&quot;$&quot;#,##0.0\ ;[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="209" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;?_);_(@_)"/>
+    <numFmt numFmtId="210" formatCode="&quot;$&quot;#,##0.000_);[Red]\(&quot;$&quot;#,##0.000\)"/>
+    <numFmt numFmtId="211" formatCode="&quot;$&quot;#,##0.00&quot;A&quot;;[Red]\(&quot;$&quot;#,##0.00\)&quot;A&quot;"/>
+    <numFmt numFmtId="212" formatCode="#,##0.0\ ;[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="213" formatCode="&quot;$&quot;#,##0.00&quot;E&quot;;[Red]\(&quot;$&quot;#,##0.00\)&quot;E&quot;"/>
+    <numFmt numFmtId="214" formatCode="_([$€-2]* #,##0.00_);_([$€-2]* \(#,##0.00\);_([$€-2]* &quot;-&quot;??_)"/>
+    <numFmt numFmtId="215" formatCode="#,##0.00;\(#,##0.00\)"/>
+    <numFmt numFmtId="216" formatCode=".%\,\(0.0%%;\t"/>
+    <numFmt numFmtId="217" formatCode="#,##0.0_);[Red]\(#,##0.0\)"/>
+    <numFmt numFmtId="218" formatCode="0.0%_);[Red]\(0.0%\)"/>
+    <numFmt numFmtId="219" formatCode="0.00_);\(0.00\);0.00_)"/>
+    <numFmt numFmtId="220" formatCode="#,##0\x"/>
+    <numFmt numFmtId="221" formatCode="&quot;TKR&quot;\ 0"/>
+    <numFmt numFmtId="222" formatCode=".%\,\(0.%%;\t"/>
+    <numFmt numFmtId="223" formatCode="&quot;$&quot;#,###.0\ \ "/>
+    <numFmt numFmtId="224" formatCode="#,##0.00\x_);[Red]\(#,##0.00\x\)"/>
+    <numFmt numFmtId="225" formatCode="#,##0.000_);\(#,##0.000\)"/>
+    <numFmt numFmtId="226" formatCode="#,##0.00\x_);[Red]\(#,##0.00\x\);&quot;--  &quot;"/>
+    <numFmt numFmtId="227" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="228" formatCode="0.0\x_);[Red]\(0.0\x\)"/>
+    <numFmt numFmtId="229" formatCode="0.0\ "/>
+    <numFmt numFmtId="230" formatCode="&quot;$&quot;#,##0.0;\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="231" formatCode="#,##0.00%_);\(#,##0.00%\)"/>
+    <numFmt numFmtId="232" formatCode="0.00\%;\-0.00\%;0.00\%"/>
+    <numFmt numFmtId="233" formatCode="0.0%\ ;\(0.0%\)"/>
+    <numFmt numFmtId="234" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="235" formatCode="&quot;$&quot;0.00\ "/>
+    <numFmt numFmtId="236" formatCode="0.0\ \ \ \ \ "/>
+    <numFmt numFmtId="237" formatCode="0.00\x;\-0.00\x;0.00\x"/>
+    <numFmt numFmtId="238" formatCode="&quot;$&quot;#,##0.000_);\(&quot;$&quot;#,##0.000\)"/>
+    <numFmt numFmtId="239" formatCode="#,##0.0_);\(#,##0.0\);_(* &quot;-&quot;_)"/>
+    <numFmt numFmtId="240" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="241" formatCode="0.00%_);[Red]\(0.00%\)"/>
+    <numFmt numFmtId="242" formatCode="#,##0.0\x_);\(#,##0.0\x\)"/>
+    <numFmt numFmtId="243" formatCode="#,##0.00\x_);\(#,##0.00\x\)"/>
+    <numFmt numFmtId="244" formatCode="###0&quot;E&quot;_)"/>
   </numFmts>
   <fonts count="105">
     <font>
@@ -1438,19 +1438,19 @@
   <cellStyleXfs count="187">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="190" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="191" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="191" fontId="10" fillId="2" borderId="0"/>
     <xf numFmtId="192" fontId="10" fillId="2" borderId="0"/>
-    <xf numFmtId="191" fontId="10" fillId="2" borderId="0"/>
     <xf numFmtId="193" fontId="10" fillId="2" borderId="0"/>
-    <xf numFmtId="194" fontId="10" fillId="2" borderId="0" applyAlignment="1">
+    <xf numFmtId="192" fontId="10" fillId="2" borderId="0"/>
+    <xf numFmtId="194" fontId="10" fillId="2" borderId="0"/>
+    <xf numFmtId="195" fontId="10" fillId="2" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="195" fontId="11" fillId="0" borderId="0"/>
+    <xf numFmtId="196" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="196" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="197" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="0"/>
@@ -1477,7 +1477,7 @@
     <xf numFmtId="0" fontId="15" fillId="20" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="0"/>
-    <xf numFmtId="197" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="198" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="38" fontId="17" fillId="0" borderId="0" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
@@ -1486,10 +1486,10 @@
       <alignment horizontal="centerContinuous"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="21" borderId="5"/>
-    <xf numFmtId="197" fontId="17" fillId="0" borderId="0" applyProtection="1">
+    <xf numFmtId="198" fontId="17" fillId="0" borderId="0" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="197" fontId="17" fillId="0" borderId="6"/>
+    <xf numFmtId="198" fontId="17" fillId="0" borderId="6"/>
     <xf numFmtId="0" fontId="21" fillId="22" borderId="7"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1507,35 +1507,35 @@
     <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="198" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="199" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
     <xf numFmtId="7" fontId="26" fillId="0" borderId="0"/>
     <xf numFmtId="5" fontId="23" fillId="0" borderId="0"/>
-    <xf numFmtId="199" fontId="13" fillId="0" borderId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="200" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="200" fontId="13" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="201" fontId="10" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="200" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="202" fontId="10" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="201" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="15" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="202" fontId="25" fillId="24" borderId="0"/>
-    <xf numFmtId="203" fontId="27" fillId="0" borderId="8"/>
+    <xf numFmtId="203" fontId="25" fillId="24" borderId="0"/>
+    <xf numFmtId="204" fontId="27" fillId="0" borderId="8"/>
     <xf numFmtId="14" fontId="28" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="204" fontId="28" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="205" fontId="28" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="205" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="206" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="8" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="6" fontId="17" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1543,48 +1543,48 @@
     <xf numFmtId="6" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="39" fontId="10" fillId="25" borderId="0"/>
     <xf numFmtId="7" fontId="10" fillId="25" borderId="0"/>
-    <xf numFmtId="206" fontId="10" fillId="25" borderId="0"/>
-    <xf numFmtId="207" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="208" fontId="10" fillId="25" borderId="0"/>
+    <xf numFmtId="207" fontId="10" fillId="25" borderId="0"/>
+    <xf numFmtId="208" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="209" fontId="10" fillId="25" borderId="0"/>
-    <xf numFmtId="210" fontId="18" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="210" fontId="10" fillId="25" borderId="0"/>
+    <xf numFmtId="211" fontId="18" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="211" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="212" fontId="18" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="212" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="213" fontId="18" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="213" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="214" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="195" fontId="10" fillId="0" borderId="10"/>
-    <xf numFmtId="214" fontId="10" fillId="2" borderId="9" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="196" fontId="10" fillId="0" borderId="10"/>
     <xf numFmtId="215" fontId="10" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="214" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="216" fontId="10" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="216" fontId="17" fillId="0" borderId="0" applyProtection="1">
+    <xf numFmtId="215" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="217" fontId="17" fillId="0" borderId="0" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="5" borderId="0"/>
-    <xf numFmtId="217" fontId="31" fillId="0" borderId="0"/>
-    <xf numFmtId="195" fontId="32" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="218" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="196" fontId="32" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="216" fontId="13" fillId="26" borderId="11"/>
+    <xf numFmtId="217" fontId="13" fillId="26" borderId="11"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="12"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="13"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="14"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0"/>
-    <xf numFmtId="216" fontId="36" fillId="0" borderId="0"/>
+    <xf numFmtId="217" fontId="36" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0"/>
-    <xf numFmtId="197" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="198" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="38" fontId="17" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
@@ -1598,7 +1598,7 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="17" fontId="39" fillId="27" borderId="0"/>
-    <xf numFmtId="218" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="219" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -1609,26 +1609,26 @@
     <xf numFmtId="173" fontId="17" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="219" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="220" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="220" fontId="10" fillId="25" borderId="0" applyAlignment="1">
+    <xf numFmtId="221" fontId="10" fillId="25" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="221" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="222" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="219" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="220" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="195" fontId="42" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="196" fontId="42" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="195" fontId="42" fillId="0" borderId="0"/>
-    <xf numFmtId="222" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="196" fontId="42" fillId="0" borderId="0"/>
+    <xf numFmtId="223" fontId="10" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="223" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="224" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="1" hidden="1"/>
@@ -1637,62 +1637,62 @@
     <xf numFmtId="37" fontId="26" fillId="0" borderId="0"/>
     <xf numFmtId="175" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="39" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="224" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="225" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
-    <xf numFmtId="225" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="226" fontId="25" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="29" borderId="17"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
-    <xf numFmtId="226" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="227" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="44" fillId="21" borderId="18"/>
-    <xf numFmtId="227" fontId="17" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="228" fontId="17" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
-    <xf numFmtId="228" fontId="10" fillId="25" borderId="0"/>
+    <xf numFmtId="229" fontId="10" fillId="25" borderId="0"/>
     <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="229" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="230" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="191" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="230" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="231" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="192" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="231" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="232" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="218" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="8" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="198" fontId="17" fillId="0" borderId="0" applyProtection="1">
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="217" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="8" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="197" fontId="17" fillId="0" borderId="0" applyProtection="1">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="216" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="38" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="193" fontId="10" fillId="2" borderId="19" applyAlignment="1">
+    <xf numFmtId="194" fontId="10" fillId="2" borderId="19" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="232" fontId="46" fillId="2" borderId="0"/>
-    <xf numFmtId="233" fontId="10" fillId="2" borderId="0"/>
+    <xf numFmtId="233" fontId="46" fillId="2" borderId="0"/>
+    <xf numFmtId="234" fontId="10" fillId="2" borderId="0"/>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="8" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="234" fontId="10" fillId="2" borderId="0" applyAlignment="1">
+    <xf numFmtId="235" fontId="10" fillId="2" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="235" fontId="10" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="236" fontId="10" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="236" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="237" fontId="12" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="216" fontId="28" fillId="0" borderId="0"/>
+    <xf numFmtId="217" fontId="28" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1700,10 +1700,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="1" hidden="1"/>
     </xf>
-    <xf numFmtId="197" fontId="17" fillId="0" borderId="0" applyProtection="1">
+    <xf numFmtId="198" fontId="17" fillId="0" borderId="0" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="237" fontId="28" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="238" fontId="28" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="38" fontId="12" fillId="0" borderId="0"/>
@@ -1721,40 +1721,40 @@
     <xf numFmtId="0" fontId="54" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="238" fontId="55" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="239" fontId="55" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="239" fontId="55" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="240" fontId="55" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="25" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="209" fontId="56" fillId="0" borderId="0"/>
-    <xf numFmtId="240" fontId="57" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="210" fontId="56" fillId="0" borderId="0"/>
+    <xf numFmtId="241" fontId="57" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="240" fontId="57" fillId="0" borderId="0"/>
-    <xf numFmtId="240" fontId="58" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="241" fontId="57" fillId="0" borderId="0"/>
+    <xf numFmtId="241" fontId="58" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="240" fontId="58" fillId="0" borderId="0" applyProtection="1">
+    <xf numFmtId="241" fontId="58" fillId="0" borderId="0" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="216" fontId="17" fillId="0" borderId="0" applyProtection="1">
+    <xf numFmtId="217" fontId="17" fillId="0" borderId="0" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="216" fontId="56" fillId="0" borderId="0"/>
+    <xf numFmtId="217" fontId="56" fillId="0" borderId="0"/>
     <xf numFmtId="49" fontId="59" fillId="0" borderId="0"/>
-    <xf numFmtId="241" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="242" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="243" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="60" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="61" fillId="1" borderId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="216" fontId="62" fillId="0" borderId="0"/>
+    <xf numFmtId="217" fontId="62" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="38" fontId="63" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1763,10 +1763,10 @@
     <xf numFmtId="0" fontId="65" fillId="0" borderId="21"/>
     <xf numFmtId="0" fontId="66" fillId="0" borderId="0"/>
     <xf numFmtId="1" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="243" fontId="26" fillId="0" borderId="0"/>
-    <xf numFmtId="237" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="244" fontId="26" fillId="0" borderId="0"/>
+    <xf numFmtId="238" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="556">
+  <cellXfs count="558">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2729,9 +2729,9 @@
     <xf numFmtId="0" fontId="100" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="101" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="102" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="244" fontId="103" fillId="34" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="190" fontId="103" fillId="34" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="104" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="244" fontId="102" fillId="35" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="190" fontId="102" fillId="35" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="102" fillId="35" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="104" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="103" fillId="34" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2744,6 +2744,8 @@
     <xf numFmtId="9" fontId="103" fillId="34" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="102" fillId="35" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="182" fontId="102" fillId="35" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="190" fontId="103" fillId="34" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="190" fontId="102" fillId="35" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="187">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4792,9 +4794,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B8:M42"/>
+  <dimension ref="B2:M43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>vengeanceaiUSC-LBOMODEL1 — ZoomInfo (GTM) LBO</t>
+        </is>
+      </c>
+    </row>
     <row r="8" ht="26.25" customHeight="1" s="244">
       <c r="B8" s="402" t="inlineStr">
         <is>
@@ -4826,21 +4835,28 @@
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>ADDED: ZoomInfo FY2025 S&amp;M → AI SDR margin model</t>
+          <t>MODEL1: LBO inputs overwritten with ZoomInfo FY2025 10-K / Q2 2026 BS + market price</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>See sheets ZI_Cover through ZI_05_Sensitivity (10-K sourced; IRR/MoM still on LBO sheet ~row 235)</t>
+          <t>Price $4.31, shares 292.3m, EBITDA $314.5m, debt $1269.9m, cash $150.1m</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>Original WSP LBO+DCF template preserved on LBO / DCF / Shares / 52wkHL tabs</t>
+          <t>Entry offer $5.39/sh (+25%); exit 8.0x; sponsor MoIC 2.97x / IRR 24.3% (illustrative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>S&amp;M AI thesis: SG&amp;A margin compressed ~500bps of revenue by Y3 in forecast (see ZI_* tabs)</t>
         </is>
       </c>
     </row>
@@ -4860,8 +4876,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:E25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="55" customWidth="1" style="244" min="2" max="2"/>
     <col width="12" customWidth="1" style="244" min="3" max="3"/>
@@ -4869,7 +4885,6 @@
     <col width="12" customWidth="1" style="244" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="539" t="inlineStr">
         <is>
@@ -4877,14 +4892,13 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="542" t="inlineStr">
         <is>
           <t>FY2025 baseline Revenue ($m)</t>
         </is>
       </c>
-      <c r="C4" s="545">
+      <c r="C4" s="557">
         <f>'ZI_01_10K_Source'!E5</f>
         <v/>
       </c>
@@ -4895,7 +4909,7 @@
           <t>FY2025 GAAP EBITDA proxy ($m)</t>
         </is>
       </c>
-      <c r="C5" s="545">
+      <c r="C5" s="557">
         <f>'ZI_01_10K_Source'!E20</f>
         <v/>
       </c>
@@ -4927,12 +4941,11 @@
           <t>Required incremental EBITDA ($m)</t>
         </is>
       </c>
-      <c r="C8" s="545">
+      <c r="C8" s="557">
         <f>C4*C7/10000</f>
         <v/>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="B10" s="542" t="inlineStr">
         <is>
@@ -4955,15 +4968,15 @@
           <t>Revenue (flat case for margin math)</t>
         </is>
       </c>
-      <c r="C11" s="545">
+      <c r="C11" s="557">
         <f>$C$4</f>
         <v/>
       </c>
-      <c r="D11" s="545">
+      <c r="D11" s="557">
         <f>$C$4</f>
         <v/>
       </c>
-      <c r="E11" s="545">
+      <c r="E11" s="557">
         <f>$C$4</f>
         <v/>
       </c>
@@ -4974,15 +4987,15 @@
           <t>Net EBITDA benefit from program</t>
         </is>
       </c>
-      <c r="C12" s="545">
+      <c r="C12" s="557">
         <f>'ZI_03_Headcount_AI'!C39</f>
         <v/>
       </c>
-      <c r="D12" s="545">
+      <c r="D12" s="557">
         <f>'ZI_03_Headcount_AI'!D39</f>
         <v/>
       </c>
-      <c r="E12" s="545">
+      <c r="E12" s="557">
         <f>'ZI_03_Headcount_AI'!E39</f>
         <v/>
       </c>
@@ -4993,15 +5006,15 @@
           <t>Run-rate benefit (ex one-time)</t>
         </is>
       </c>
-      <c r="C13" s="545">
+      <c r="C13" s="557">
         <f>'ZI_03_Headcount_AI'!C40</f>
         <v/>
       </c>
-      <c r="D13" s="545">
+      <c r="D13" s="557">
         <f>'ZI_03_Headcount_AI'!D40</f>
         <v/>
       </c>
-      <c r="E13" s="545">
+      <c r="E13" s="557">
         <f>'ZI_03_Headcount_AI'!E40</f>
         <v/>
       </c>
@@ -5012,15 +5025,15 @@
           <t>Pro forma EBITDA</t>
         </is>
       </c>
-      <c r="C14" s="545">
+      <c r="C14" s="557">
         <f>$C$5+C12</f>
         <v/>
       </c>
-      <c r="D14" s="545">
+      <c r="D14" s="557">
         <f>$C$5+D12</f>
         <v/>
       </c>
-      <c r="E14" s="545">
+      <c r="E14" s="557">
         <f>$C$5+E12</f>
         <v/>
       </c>
@@ -5050,15 +5063,15 @@
           <t>Margin expansion (bps)</t>
         </is>
       </c>
-      <c r="C16" s="545">
+      <c r="C16" s="557">
         <f>(C15-$C$6)*10000</f>
         <v/>
       </c>
-      <c r="D16" s="545">
+      <c r="D16" s="557">
         <f>(D15-$C$6)*10000</f>
         <v/>
       </c>
-      <c r="E16" s="545">
+      <c r="E16" s="557">
         <f>(E15-$C$6)*10000</f>
         <v/>
       </c>
@@ -5069,15 +5082,15 @@
           <t>Run-rate expansion (bps)</t>
         </is>
       </c>
-      <c r="C17" s="545">
+      <c r="C17" s="557">
         <f>(C13/$C$4)*10000</f>
         <v/>
       </c>
-      <c r="D17" s="545">
+      <c r="D17" s="557">
         <f>(D13/$C$4)*10000</f>
         <v/>
       </c>
-      <c r="E17" s="545">
+      <c r="E17" s="557">
         <f>(E13/$C$4)*10000</f>
         <v/>
       </c>
@@ -5101,7 +5114,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="B20" s="542" t="inlineStr">
         <is>
@@ -5126,15 +5138,15 @@
           <t>PF S&amp;M $ (baseline − SDR save + AI/oversight)</t>
         </is>
       </c>
-      <c r="C22" s="545">
+      <c r="C22" s="557">
         <f>'ZI_01_10K_Source'!E6-'ZI_03_Headcount_AI'!C34+'ZI_03_Headcount_AI'!C35+'ZI_03_Headcount_AI'!C36</f>
         <v/>
       </c>
-      <c r="D22" s="545">
+      <c r="D22" s="557">
         <f>'ZI_01_10K_Source'!E6-'ZI_03_Headcount_AI'!D34+'ZI_03_Headcount_AI'!D35+'ZI_03_Headcount_AI'!D36</f>
         <v/>
       </c>
-      <c r="E22" s="545">
+      <c r="E22" s="557">
         <f>'ZI_01_10K_Source'!E6-'ZI_03_Headcount_AI'!E34+'ZI_03_Headcount_AI'!E35+'ZI_03_Headcount_AI'!E36</f>
         <v/>
       </c>
@@ -5158,7 +5170,6 @@
         <v/>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
@@ -5177,8 +5188,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:H20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" style="244" min="2" max="2"/>
     <col width="10" customWidth="1" style="244" min="3" max="3"/>
@@ -5189,7 +5200,6 @@
     <col width="10" customWidth="1" style="244" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="539" t="inlineStr">
         <is>
@@ -5204,7 +5214,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="542" t="inlineStr">
         <is>
@@ -5222,7 +5231,7 @@
           <t>SDR cost $k</t>
         </is>
       </c>
-      <c r="C6" s="545">
+      <c r="C6" s="557">
         <f>'ZI_03_Headcount_AI'!C8</f>
         <v/>
       </c>
@@ -5244,7 +5253,7 @@
           <t>Oversight $k</t>
         </is>
       </c>
-      <c r="C8" s="545">
+      <c r="C8" s="557">
         <f>'ZI_03_Headcount_AI'!C15</f>
         <v/>
       </c>
@@ -5255,12 +5264,11 @@
           <t>Revenue $m</t>
         </is>
       </c>
-      <c r="C9" s="545">
+      <c r="C9" s="557">
         <f>'ZI_01_10K_Source'!E5</f>
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
@@ -5460,15 +5468,13 @@
         <v/>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
     <row r="20">
       <c r="B20" s="542" t="inlineStr">
         <is>
           <t>Base case Y3 run-rate bps (from bridge)</t>
         </is>
       </c>
-      <c r="C20" s="545">
+      <c r="C20" s="557">
         <f>'ZI_04_EBITDA_Bridge'!E17</f>
         <v/>
       </c>
@@ -5485,7 +5491,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A2:R393"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="1.7109375" customWidth="1" style="244" min="1" max="1"/>
     <col width="44.140625" customWidth="1" style="244" min="2" max="2"/>
@@ -5498,7 +5504,7 @@
     <row r="2" ht="27" customHeight="1" s="244" thickBot="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Leveraged buyout model for BMC</t>
+          <t>Leveraged buyout model for ZoomInfo (GTM) — vengeanceaiUSC-LBOMODEL1</t>
         </is>
       </c>
       <c r="C2" s="305" t="n"/>
@@ -5548,7 +5554,7 @@
       </c>
       <c r="D6" s="378" t="inlineStr">
         <is>
-          <t>BMC</t>
+          <t>ZoomInfo Technologies Inc.</t>
         </is>
       </c>
     </row>
@@ -5560,7 +5566,7 @@
       </c>
       <c r="D7" s="378" t="inlineStr">
         <is>
-          <t>BMC</t>
+          <t>GTM</t>
         </is>
       </c>
       <c r="F7" s="100" t="inlineStr">
@@ -5569,7 +5575,7 @@
         </is>
       </c>
       <c r="H7" s="406" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="407" t="n">
         <v>1</v>
@@ -5585,7 +5591,7 @@
         </is>
       </c>
       <c r="D8" s="135" t="n">
-        <v>45.42</v>
+        <v>4.31</v>
       </c>
       <c r="H8" s="409" t="inlineStr">
         <is>
@@ -5610,7 +5616,7 @@
         </is>
       </c>
       <c r="D9" s="365" t="n">
-        <v>41400</v>
+        <v>46246</v>
       </c>
     </row>
     <row r="10">
@@ -5630,13 +5636,13 @@
         </is>
       </c>
       <c r="H10" s="140" t="n">
-        <v>882.7000000000003</v>
+        <v>314.5</v>
       </c>
       <c r="I10" s="140" t="n">
-        <v>882.7000000000003</v>
+        <v>314.5</v>
       </c>
       <c r="J10" s="140" t="n">
-        <v>882.7000000000003</v>
+        <v>314.5</v>
       </c>
     </row>
     <row r="11">
@@ -5646,13 +5652,13 @@
         </is>
       </c>
       <c r="H11" s="411" t="n">
-        <v>7.325281805823042</v>
+        <v>8.57</v>
       </c>
       <c r="I11" s="412" t="n">
-        <v>7.3</v>
+        <v>8.57</v>
       </c>
       <c r="J11" s="411" t="n">
-        <v>7.325281805823042</v>
+        <v>8.57</v>
       </c>
     </row>
     <row r="12">
@@ -5669,13 +5675,13 @@
         </is>
       </c>
       <c r="H12" s="57" t="n">
-        <v>6466.026250000001</v>
+        <v>2694.6</v>
       </c>
       <c r="I12" s="57" t="n">
-        <v>6443.710000000002</v>
+        <v>2694.6</v>
       </c>
       <c r="J12" s="57" t="n">
-        <v>6466.026250000001</v>
+        <v>2694.6</v>
       </c>
     </row>
     <row r="13">
@@ -5685,7 +5691,7 @@
         </is>
       </c>
       <c r="D13" s="413" t="n">
-        <v>882.7000000000003</v>
+        <v>314.5</v>
       </c>
     </row>
     <row r="14">
@@ -5695,7 +5701,7 @@
         </is>
       </c>
       <c r="D14" s="228" t="n">
-        <v>-1306</v>
+        <v>-1269.9</v>
       </c>
       <c r="F14" s="159" t="inlineStr">
         <is>
@@ -5703,13 +5709,13 @@
         </is>
       </c>
       <c r="H14" s="140" t="n">
-        <v>-1306</v>
+        <v>-1269.9</v>
       </c>
       <c r="I14" s="140" t="n">
-        <v>-1306</v>
+        <v>-1269.9</v>
       </c>
       <c r="J14" s="140" t="n">
-        <v>-1306</v>
+        <v>-1269.9</v>
       </c>
     </row>
     <row r="15">
@@ -5719,7 +5725,7 @@
         </is>
       </c>
       <c r="D15" s="228" t="n">
-        <v>1581.9</v>
+        <v>150.1</v>
       </c>
       <c r="F15" s="159" t="inlineStr">
         <is>
@@ -5727,13 +5733,13 @@
         </is>
       </c>
       <c r="H15" s="140" t="n">
-        <v>1581.9</v>
+        <v>150.1</v>
       </c>
       <c r="I15" s="140" t="n">
-        <v>1581.9</v>
+        <v>150.1</v>
       </c>
       <c r="J15" s="140" t="n">
-        <v>1581.9</v>
+        <v>150.1</v>
       </c>
     </row>
     <row r="16">
@@ -5743,7 +5749,7 @@
         </is>
       </c>
       <c r="D16" s="228" t="n">
-        <v>180</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -5753,7 +5759,7 @@
         </is>
       </c>
       <c r="D17" s="412" t="n">
-        <v>7.3</v>
+        <v>8</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
@@ -5761,13 +5767,13 @@
         </is>
       </c>
       <c r="H17" s="57" t="n">
-        <v>6741.92625</v>
+        <v>1574.8</v>
       </c>
       <c r="I17" s="57" t="n">
-        <v>6719.610000000002</v>
+        <v>1574.8</v>
       </c>
       <c r="J17" s="57" t="n">
-        <v>6741.92625</v>
+        <v>1574.8</v>
       </c>
     </row>
     <row r="18">
@@ -5778,13 +5784,13 @@
         </is>
       </c>
       <c r="H18" s="415" t="n">
-        <v>145.7713783783784</v>
+        <v>292.312</v>
       </c>
       <c r="I18" s="413" t="n">
-        <v>145.7713783783784</v>
+        <v>292.312</v>
       </c>
       <c r="J18" s="413" t="n">
-        <v>145.7713783783784</v>
+        <v>292.312</v>
       </c>
       <c r="K18" s="416" t="n"/>
       <c r="L18" s="416" t="n"/>
@@ -5807,7 +5813,7 @@
         </is>
       </c>
       <c r="D20" s="417" t="n">
-        <v>6741.92625</v>
+        <v>1574.8</v>
       </c>
       <c r="E20" s="418" t="n"/>
       <c r="F20" s="3" t="inlineStr">
@@ -5816,13 +5822,13 @@
         </is>
       </c>
       <c r="H20" s="307" t="n">
-        <v>46.25</v>
+        <v>5.3875</v>
       </c>
       <c r="I20" s="307" t="n">
-        <v>46.09690924756112</v>
+        <v>5.3875</v>
       </c>
       <c r="J20" s="366" t="n">
-        <v>46.25</v>
+        <v>5.3875</v>
       </c>
       <c r="K20" s="416" t="n"/>
       <c r="L20" s="416" t="n"/>
@@ -5834,7 +5840,7 @@
         </is>
       </c>
       <c r="D21" s="417" t="n">
-        <v>1306</v>
+        <v>1269.9</v>
       </c>
       <c r="E21" s="418" t="n"/>
       <c r="F21" s="158" t="inlineStr">
@@ -5843,13 +5849,13 @@
         </is>
       </c>
       <c r="H21" s="418" t="n">
-        <v>0.01827388815499775</v>
+        <v>0.25</v>
       </c>
       <c r="I21" s="418" t="n">
-        <v>0.01490332997712729</v>
+        <v>0.25</v>
       </c>
       <c r="J21" s="418" t="n">
-        <v>0.01827388815499775</v>
+        <v>0.25</v>
       </c>
       <c r="K21" s="416" t="n"/>
       <c r="L21" s="416" t="n"/>
@@ -5861,7 +5867,7 @@
         </is>
       </c>
       <c r="D22" s="419" t="n">
-        <v>204.52769</v>
+        <v>31.5</v>
       </c>
       <c r="H22" s="158" t="n"/>
       <c r="J22" s="420" t="n"/>
@@ -5875,7 +5881,7 @@
         </is>
       </c>
       <c r="D23" s="421" t="n">
-        <v>8252.453940000001</v>
+        <v>2876.2</v>
       </c>
       <c r="H23" s="158" t="n"/>
       <c r="J23" s="420" t="n"/>
@@ -5947,10 +5953,10 @@
         </is>
       </c>
       <c r="C27" s="422" t="n">
-        <v>1.588195309844794</v>
+        <v>0.318</v>
       </c>
       <c r="D27" s="417" t="n">
-        <v>1401.9</v>
+        <v>100.1</v>
       </c>
       <c r="F27" s="100" t="inlineStr">
         <is>
@@ -5995,10 +6001,10 @@
         </is>
       </c>
       <c r="C29" s="427" t="n">
-        <v>3.27</v>
+        <v>2.5</v>
       </c>
       <c r="D29" s="417" t="n">
-        <v>2886.429000000001</v>
+        <v>786.2</v>
       </c>
       <c r="F29" s="34" t="inlineStr">
         <is>
@@ -6025,10 +6031,10 @@
         </is>
       </c>
       <c r="C30" s="427" t="n">
-        <v>0.76</v>
+        <v>1.5</v>
       </c>
       <c r="D30" s="417" t="n">
-        <v>670.8520000000002</v>
+        <v>471.8</v>
       </c>
       <c r="F30" s="34" t="inlineStr">
         <is>
@@ -6057,10 +6063,10 @@
         </is>
       </c>
       <c r="C31" s="427" t="n">
-        <v>1.85</v>
+        <v>1</v>
       </c>
       <c r="D31" s="417" t="n">
-        <v>1632.995000000001</v>
+        <v>314.5</v>
       </c>
       <c r="F31" s="34" t="inlineStr">
         <is>
@@ -6132,7 +6138,7 @@
         </is>
       </c>
       <c r="H33" s="421" t="n">
-        <v>69.68916500000003</v>
+        <v>23.6</v>
       </c>
       <c r="I33" s="202" t="n"/>
       <c r="J33" s="417" t="n">
@@ -6164,10 +6170,10 @@
         </is>
       </c>
       <c r="C35" s="422" t="n">
-        <v>1.880908507986857</v>
+        <v>3.827</v>
       </c>
       <c r="D35" s="428" t="n">
-        <v>1660.277939999999</v>
+        <v>1203.6</v>
       </c>
       <c r="F35" s="34" t="n"/>
       <c r="G35" s="296" t="inlineStr">
@@ -6190,10 +6196,10 @@
         </is>
       </c>
       <c r="C36" s="430" t="n">
-        <v>9.349103817831651</v>
+        <v>9.145</v>
       </c>
       <c r="D36" s="421" t="n">
-        <v>8252.453940000001</v>
+        <v>2876.2</v>
       </c>
       <c r="F36" s="332" t="inlineStr">
         <is>
@@ -6204,10 +6210,9 @@
         <v>0.02</v>
       </c>
       <c r="H36" s="421" t="n">
-        <v>134.838525</v>
-      </c>
-    </row>
-    <row r="37"/>
+        <v>31.5</v>
+      </c>
+    </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -6235,28 +6240,28 @@
         </is>
       </c>
       <c r="C39" s="270" t="n">
-        <v>2011</v>
+        <v>2023</v>
       </c>
       <c r="D39" s="270" t="n">
-        <v>2012</v>
+        <v>2024</v>
       </c>
       <c r="E39" s="431" t="n">
-        <v>2013</v>
+        <v>2025</v>
       </c>
       <c r="F39" s="157" t="n">
-        <v>2014</v>
+        <v>2026</v>
       </c>
       <c r="G39" s="157" t="n">
-        <v>2015</v>
+        <v>2027</v>
       </c>
       <c r="H39" s="157" t="n">
-        <v>2016</v>
+        <v>2028</v>
       </c>
       <c r="I39" s="157" t="n">
-        <v>2017</v>
+        <v>2029</v>
       </c>
       <c r="J39" s="157" t="n">
-        <v>2018</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="40">
@@ -6266,28 +6271,28 @@
         </is>
       </c>
       <c r="C40" s="19" t="n">
-        <v>40633</v>
+        <v>45291</v>
       </c>
       <c r="D40" s="19" t="n">
-        <v>40999</v>
+        <v>45657</v>
       </c>
       <c r="E40" s="19" t="n">
-        <v>41364</v>
+        <v>46022</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>41729</v>
+        <v>46387</v>
       </c>
       <c r="G40" s="20" t="n">
-        <v>42094</v>
+        <v>46752</v>
       </c>
       <c r="H40" s="20" t="n">
-        <v>42460</v>
+        <v>47118</v>
       </c>
       <c r="I40" s="20" t="n">
-        <v>42825</v>
+        <v>47483</v>
       </c>
       <c r="J40" s="20" t="n">
-        <v>43190</v>
+        <v>47848</v>
       </c>
     </row>
     <row r="41">
@@ -6308,28 +6313,28 @@
         </is>
       </c>
       <c r="C42" s="432" t="n">
-        <v>2065.3</v>
+        <v>1239.5</v>
       </c>
       <c r="D42" s="432" t="n">
-        <v>2172</v>
+        <v>1214.3</v>
       </c>
       <c r="E42" s="432" t="n">
-        <v>2201.4</v>
+        <v>1249.5</v>
       </c>
       <c r="F42" s="413" t="n">
-        <v>2278.449</v>
+        <v>1299.5</v>
       </c>
       <c r="G42" s="413" t="n">
-        <v>2403.763695</v>
+        <v>1364.5</v>
       </c>
       <c r="H42" s="413" t="n">
-        <v>2547.9895167</v>
+        <v>1432.7</v>
       </c>
       <c r="I42" s="413" t="n">
-        <v>2675.388992535</v>
+        <v>1490</v>
       </c>
       <c r="J42" s="413" t="n">
-        <v>2803.807664176681</v>
+        <v>1534.7</v>
       </c>
     </row>
     <row r="43">
@@ -6339,28 +6344,28 @@
         </is>
       </c>
       <c r="C43" s="432" t="n">
-        <v>-485.2</v>
+        <v>-200.4</v>
       </c>
       <c r="D43" s="432" t="n">
-        <v>-568.9</v>
+        <v>-211.4</v>
       </c>
       <c r="E43" s="432" t="n">
-        <v>-592</v>
+        <v>-220.5</v>
       </c>
       <c r="F43" s="413" t="n">
-        <v>-581.5921997023499</v>
+        <v>-222.8</v>
       </c>
       <c r="G43" s="413" t="n">
-        <v>-601.5609522109792</v>
+        <v>-234</v>
       </c>
       <c r="H43" s="413" t="n">
-        <v>-624.914661760138</v>
+        <v>-245.7</v>
       </c>
       <c r="I43" s="413" t="n">
-        <v>-642.7834498854697</v>
+        <v>-255.5</v>
       </c>
       <c r="J43" s="413" t="n">
-        <v>-659.618017159089</v>
+        <v>-263.2</v>
       </c>
     </row>
     <row r="44">
@@ -6370,28 +6375,28 @@
         </is>
       </c>
       <c r="C44" s="433" t="n">
-        <v>1580.1</v>
+        <v>1039.1</v>
       </c>
       <c r="D44" s="433" t="n">
-        <v>1603.1</v>
+        <v>1002.9</v>
       </c>
       <c r="E44" s="433" t="n">
-        <v>1609.4</v>
+        <v>1029</v>
       </c>
       <c r="F44" s="433" t="n">
-        <v>1696.85680029765</v>
+        <v>1076.7</v>
       </c>
       <c r="G44" s="433" t="n">
-        <v>1802.202742789021</v>
+        <v>1130.5</v>
       </c>
       <c r="H44" s="433" t="n">
-        <v>1923.074854939862</v>
+        <v>1187</v>
       </c>
       <c r="I44" s="433" t="n">
-        <v>2032.605542649531</v>
+        <v>1234.5</v>
       </c>
       <c r="J44" s="433" t="n">
-        <v>2144.189647017592</v>
+        <v>1271.5</v>
       </c>
     </row>
     <row r="45">
@@ -6401,28 +6406,28 @@
         </is>
       </c>
       <c r="C45" s="432" t="n">
-        <v>-181.6</v>
+        <v>-191.5</v>
       </c>
       <c r="D45" s="432" t="n">
-        <v>-165.2</v>
+        <v>-196.1</v>
       </c>
       <c r="E45" s="432" t="n">
-        <v>-174.6</v>
+        <v>-182</v>
       </c>
       <c r="F45" s="413" t="n">
-        <v>-184.7831333486259</v>
+        <v>-189.3</v>
       </c>
       <c r="G45" s="413" t="n">
-        <v>-194.9462056828004</v>
+        <v>-198.7</v>
       </c>
       <c r="H45" s="413" t="n">
-        <v>-206.6429780237684</v>
+        <v>-208.7</v>
       </c>
       <c r="I45" s="413" t="n">
-        <v>-216.9751269249568</v>
+        <v>-217</v>
       </c>
       <c r="J45" s="413" t="n">
-        <v>-227.3899330173548</v>
+        <v>-223.5</v>
       </c>
     </row>
     <row r="46">
@@ -6432,28 +6437,28 @@
         </is>
       </c>
       <c r="C46" s="432" t="n">
-        <v>-865.6999999999999</v>
+        <v>-588.1</v>
       </c>
       <c r="D46" s="432" t="n">
-        <v>-894</v>
+        <v>-709.4</v>
       </c>
       <c r="E46" s="432" t="n">
-        <v>-969.3999999999999</v>
+        <v>-621.3</v>
       </c>
       <c r="F46" s="413" t="n">
-        <v>-965.3960306852802</v>
+        <v>-620.2</v>
       </c>
       <c r="G46" s="413" t="n">
-        <v>-994.4551754229706</v>
+        <v>-630.7</v>
       </c>
       <c r="H46" s="413" t="n">
-        <v>-1028.642590781349</v>
+        <v>-640.7</v>
       </c>
       <c r="I46" s="413" t="n">
-        <v>-1053.320830395066</v>
+        <v>-658.9</v>
       </c>
       <c r="J46" s="413" t="n">
-        <v>-1075.842153612263</v>
+        <v>-678.7</v>
       </c>
     </row>
     <row r="47">
@@ -6466,19 +6471,19 @@
       <c r="D47" s="432" t="n"/>
       <c r="E47" s="432" t="n"/>
       <c r="F47" s="413" t="n">
-        <v>-52.99732208333334</v>
+        <v>0</v>
       </c>
       <c r="G47" s="413" t="n">
-        <v>-52.99732208333334</v>
+        <v>0</v>
       </c>
       <c r="H47" s="413" t="n">
-        <v>-52.99732208333334</v>
+        <v>0</v>
       </c>
       <c r="I47" s="413" t="n">
-        <v>-52.99732208333334</v>
+        <v>0</v>
       </c>
       <c r="J47" s="413" t="n">
-        <v>-52.99732208333334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -6488,28 +6493,28 @@
         </is>
       </c>
       <c r="C48" s="433" t="n">
-        <v>532.8000000000003</v>
+        <v>259.5</v>
       </c>
       <c r="D48" s="433" t="n">
-        <v>543.8999999999999</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="E48" s="433" t="n">
-        <v>465.4000000000003</v>
+        <v>225.7</v>
       </c>
       <c r="F48" s="433" t="n">
-        <v>493.6803141804108</v>
+        <v>267.2</v>
       </c>
       <c r="G48" s="433" t="n">
-        <v>559.8040395999167</v>
+        <v>301</v>
       </c>
       <c r="H48" s="433" t="n">
-        <v>634.7919640514119</v>
+        <v>337.6</v>
       </c>
       <c r="I48" s="433" t="n">
-        <v>709.3122632461741</v>
+        <v>358.5</v>
       </c>
       <c r="J48" s="433" t="n">
-        <v>787.9602383046408</v>
+        <v>369.3</v>
       </c>
       <c r="K48" s="140" t="n"/>
     </row>
@@ -6520,28 +6525,28 @@
         </is>
       </c>
       <c r="C49" s="432" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D49" s="432" t="n">
-        <v>10.6</v>
+        <v>0</v>
       </c>
       <c r="E49" s="432" t="n">
-        <v>8.300000000000001</v>
+        <v>0</v>
       </c>
       <c r="F49" s="417" t="n">
-        <v>0.9286713286713288</v>
+        <v>0</v>
       </c>
       <c r="G49" s="417" t="n">
-        <v>0.9286713286713288</v>
+        <v>0</v>
       </c>
       <c r="H49" s="417" t="n">
-        <v>0.9286713286713288</v>
+        <v>0</v>
       </c>
       <c r="I49" s="417" t="n">
-        <v>0.9286713286713288</v>
+        <v>0</v>
       </c>
       <c r="J49" s="417" t="n">
-        <v>0.9286713286713283</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -6551,28 +6556,28 @@
         </is>
       </c>
       <c r="C50" s="432" t="n">
-        <v>-19.8</v>
+        <v>-45.2</v>
       </c>
       <c r="D50" s="432" t="n">
-        <v>-23.3</v>
+        <v>-39.3</v>
       </c>
       <c r="E50" s="432" t="n">
-        <v>-47.8</v>
+        <v>-42.6</v>
       </c>
       <c r="F50" s="417" t="n">
-        <v>-296.9412607964802</v>
+        <v>-110.1</v>
       </c>
       <c r="G50" s="417" t="n">
-        <v>-275.9548849256559</v>
+        <v>-96.90000000000001</v>
       </c>
       <c r="H50" s="417" t="n">
-        <v>-256.9076268895943</v>
+        <v>-83.7</v>
       </c>
       <c r="I50" s="417" t="n">
-        <v>-230.9705847706274</v>
+        <v>-70.40000000000001</v>
       </c>
       <c r="J50" s="417" t="n">
-        <v>-192.5062463049772</v>
+        <v>-57.2</v>
       </c>
     </row>
     <row r="51">
@@ -6582,13 +6587,13 @@
         </is>
       </c>
       <c r="C51" s="432" t="n">
-        <v>3.3</v>
+        <v>0</v>
       </c>
       <c r="D51" s="432" t="n">
-        <v>-1.2</v>
+        <v>0</v>
       </c>
       <c r="E51" s="432" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F51" s="432" t="n">
         <v>0</v>
@@ -6613,28 +6618,28 @@
         </is>
       </c>
       <c r="C52" s="433" t="n">
-        <v>531.3000000000003</v>
+        <v>214.3</v>
       </c>
       <c r="D52" s="433" t="n">
-        <v>529.9999999999999</v>
+        <v>58.1</v>
       </c>
       <c r="E52" s="433" t="n">
-        <v>427.9000000000003</v>
+        <v>183.1</v>
       </c>
       <c r="F52" s="433" t="n">
-        <v>197.6677247126019</v>
+        <v>157.1</v>
       </c>
       <c r="G52" s="433" t="n">
-        <v>284.7778260029322</v>
+        <v>204.2</v>
       </c>
       <c r="H52" s="433" t="n">
-        <v>378.813008490489</v>
+        <v>253.9</v>
       </c>
       <c r="I52" s="433" t="n">
-        <v>479.2703498042181</v>
+        <v>288.1</v>
       </c>
       <c r="J52" s="433" t="n">
-        <v>596.382663328335</v>
+        <v>312.1</v>
       </c>
     </row>
     <row r="53">
@@ -6644,28 +6649,28 @@
         </is>
       </c>
       <c r="C53" s="432" t="n">
-        <v>-75.09999999999999</v>
+        <v>-281.5</v>
       </c>
       <c r="D53" s="432" t="n">
-        <v>-129</v>
+        <v>-2.2</v>
       </c>
       <c r="E53" s="432" t="n">
-        <v>-96.90000000000001</v>
+        <v>-70.09999999999999</v>
       </c>
       <c r="F53" s="413" t="n">
-        <v>-44.76280094566748</v>
+        <v>-33</v>
       </c>
       <c r="G53" s="413" t="n">
-        <v>-64.48929969545246</v>
+        <v>-42.9</v>
       </c>
       <c r="H53" s="413" t="n">
-        <v>-85.78401617837896</v>
+        <v>-53.3</v>
       </c>
       <c r="I53" s="413" t="n">
-        <v>-108.5330612199783</v>
+        <v>-60.5</v>
       </c>
       <c r="J53" s="413" t="n">
-        <v>-135.0537043152971</v>
+        <v>-65.5</v>
       </c>
     </row>
     <row r="54">
@@ -6675,28 +6680,28 @@
         </is>
       </c>
       <c r="C54" s="433" t="n">
-        <v>456.2000000000003</v>
+        <v>-67.2</v>
       </c>
       <c r="D54" s="433" t="n">
-        <v>400.9999999999999</v>
+        <v>55.9</v>
       </c>
       <c r="E54" s="433" t="n">
-        <v>331.0000000000003</v>
+        <v>113</v>
       </c>
       <c r="F54" s="433" t="n">
-        <v>152.9049237669344</v>
+        <v>124.1</v>
       </c>
       <c r="G54" s="433" t="n">
-        <v>220.2885263074797</v>
+        <v>161.3</v>
       </c>
       <c r="H54" s="433" t="n">
-        <v>293.02899231211</v>
+        <v>200.6</v>
       </c>
       <c r="I54" s="433" t="n">
-        <v>370.7372885842398</v>
+        <v>227.6</v>
       </c>
       <c r="J54" s="433" t="n">
-        <v>461.3289590130379</v>
+        <v>246.5</v>
       </c>
     </row>
     <row r="55">
@@ -6731,28 +6736,28 @@
         </is>
       </c>
       <c r="C57" s="421" t="n">
-        <v>532.8000000000003</v>
+        <v>259.5</v>
       </c>
       <c r="D57" s="421" t="n">
-        <v>543.8999999999999</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="E57" s="421" t="n">
-        <v>465.4000000000003</v>
+        <v>225.7</v>
       </c>
       <c r="F57" s="421" t="n">
-        <v>493.6803141804108</v>
+        <v>267.2</v>
       </c>
       <c r="G57" s="421" t="n">
-        <v>559.8040395999167</v>
+        <v>301</v>
       </c>
       <c r="H57" s="421" t="n">
-        <v>634.7919640514119</v>
+        <v>337.6</v>
       </c>
       <c r="I57" s="421" t="n">
-        <v>709.3122632461741</v>
+        <v>358.5</v>
       </c>
       <c r="J57" s="421" t="n">
-        <v>787.9602383046408</v>
+        <v>369.3</v>
       </c>
     </row>
     <row r="58">
@@ -6762,28 +6767,28 @@
         </is>
       </c>
       <c r="C58" s="432" t="n">
-        <v>190</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="D58" s="432" t="n">
-        <v>224.6</v>
+        <v>85.7</v>
       </c>
       <c r="E58" s="432" t="n">
-        <v>229</v>
+        <v>88.8</v>
       </c>
       <c r="F58" s="417" t="n">
-        <v>223.946868228773</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="G58" s="417" t="n">
-        <v>220.6010317460318</v>
+        <v>97</v>
       </c>
       <c r="H58" s="417" t="n">
-        <v>222.400781053162</v>
+        <v>101.8</v>
       </c>
       <c r="I58" s="417" t="n">
-        <v>224.1937314184933</v>
+        <v>105.9</v>
       </c>
       <c r="J58" s="417" t="n">
-        <v>223</v>
+        <v>109.1</v>
       </c>
     </row>
     <row r="59">
@@ -6796,19 +6801,19 @@
       <c r="D59" s="432" t="n"/>
       <c r="E59" s="432" t="n"/>
       <c r="F59" s="413" t="n">
-        <v>52.99732208333334</v>
+        <v>0</v>
       </c>
       <c r="G59" s="413" t="n">
-        <v>52.99732208333334</v>
+        <v>0</v>
       </c>
       <c r="H59" s="413" t="n">
-        <v>52.99732208333334</v>
+        <v>0</v>
       </c>
       <c r="I59" s="413" t="n">
-        <v>52.99732208333334</v>
+        <v>0</v>
       </c>
       <c r="J59" s="413" t="n">
-        <v>52.99732208333334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -6818,28 +6823,28 @@
         </is>
       </c>
       <c r="C60" s="432" t="n">
-        <v>106.5</v>
+        <v>167.6</v>
       </c>
       <c r="D60" s="432" t="n">
-        <v>127.2</v>
+        <v>138</v>
       </c>
       <c r="E60" s="432" t="n">
-        <v>147.4</v>
+        <v>116.2</v>
       </c>
       <c r="F60" s="417" t="n">
-        <v>161.0547368274718</v>
+        <v>120.8</v>
       </c>
       <c r="G60" s="417" t="n">
-        <v>162.0820911651659</v>
+        <v>126.9</v>
       </c>
       <c r="H60" s="417" t="n">
-        <v>163.6976202897424</v>
+        <v>133.2</v>
       </c>
       <c r="I60" s="417" t="n">
-        <v>163.5682893160696</v>
+        <v>138.6</v>
       </c>
       <c r="J60" s="417" t="n">
-        <v>162.9165586144626</v>
+        <v>142.7</v>
       </c>
     </row>
     <row r="61">
@@ -6849,22 +6854,22 @@
         </is>
       </c>
       <c r="C61" s="432" t="n">
-        <v>14.3</v>
+        <v>0</v>
       </c>
       <c r="D61" s="432" t="n">
-        <v>10.8</v>
+        <v>0</v>
       </c>
       <c r="E61" s="432" t="n">
-        <v>40.9</v>
+        <v>0</v>
       </c>
       <c r="F61" s="432" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="G61" s="432" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H61" s="432" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I61" s="432" t="n">
         <v>0</v>
@@ -6880,28 +6885,28 @@
         </is>
       </c>
       <c r="C62" s="433" t="n">
-        <v>843.6000000000003</v>
+        <v>340.1</v>
       </c>
       <c r="D62" s="433" t="n">
-        <v>906.4999999999999</v>
+        <v>183.1</v>
       </c>
       <c r="E62" s="433" t="n">
-        <v>882.7000000000003</v>
+        <v>314.5</v>
       </c>
       <c r="F62" s="433" t="n">
-        <v>947.6792413199889</v>
+        <v>359.6</v>
       </c>
       <c r="G62" s="433" t="n">
-        <v>1000.484484594448</v>
+        <v>398</v>
       </c>
       <c r="H62" s="433" t="n">
-        <v>1078.88768747765</v>
+        <v>439.4</v>
       </c>
       <c r="I62" s="433" t="n">
-        <v>1150.07160606407</v>
+        <v>464.4</v>
       </c>
       <c r="J62" s="433" t="n">
-        <v>1226.874119002437</v>
+        <v>478.4</v>
       </c>
     </row>
     <row r="63">
@@ -6928,25 +6933,25 @@
       </c>
       <c r="C65" s="418" t="n"/>
       <c r="D65" s="418" t="n">
-        <v>0.05166319663002938</v>
+        <v>-0.0203</v>
       </c>
       <c r="E65" s="418" t="n">
-        <v>0.01353591160221002</v>
+        <v>0.029</v>
       </c>
       <c r="F65" s="424" t="n">
-        <v>0.035</v>
+        <v>0.04</v>
       </c>
       <c r="G65" s="424" t="n">
-        <v>0.055</v>
+        <v>0.05</v>
       </c>
       <c r="H65" s="424" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="I65" s="424" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="J65" s="424" t="n">
-        <v>0.048</v>
+        <v>0.03</v>
       </c>
       <c r="K65" s="424" t="n"/>
     </row>
@@ -6957,28 +6962,28 @@
         </is>
       </c>
       <c r="C66" s="418" t="n">
-        <v>0.7650704498135864</v>
+        <v>0.8383</v>
       </c>
       <c r="D66" s="418" t="n">
-        <v>0.7380755064456721</v>
+        <v>0.8259</v>
       </c>
       <c r="E66" s="418" t="n">
-        <v>0.7310802216771146</v>
+        <v>0.8235</v>
       </c>
       <c r="F66" s="434" t="n">
-        <v>0.7447420593121242</v>
+        <v>0.8285</v>
       </c>
       <c r="G66" s="434" t="n">
-        <v>0.7497420593121242</v>
+        <v>0.8285</v>
       </c>
       <c r="H66" s="434" t="n">
-        <v>0.7547420593121242</v>
+        <v>0.8285</v>
       </c>
       <c r="I66" s="434" t="n">
-        <v>0.7597420593121242</v>
+        <v>0.8285</v>
       </c>
       <c r="J66" s="434" t="n">
-        <v>0.7647420593121242</v>
+        <v>0.8285</v>
       </c>
       <c r="K66" s="424" t="n">
         <v>0.005</v>
@@ -6991,28 +6996,28 @@
         </is>
       </c>
       <c r="C67" s="418" t="n">
-        <v>0.08792911441437078</v>
+        <v>0.1545</v>
       </c>
       <c r="D67" s="418" t="n">
-        <v>0.07605893186003683</v>
+        <v>0.1615</v>
       </c>
       <c r="E67" s="418" t="n">
-        <v>0.07931316434995911</v>
+        <v>0.1457</v>
       </c>
       <c r="F67" s="434" t="n">
-        <v>0.08110040354145558</v>
+        <v>0.1457</v>
       </c>
       <c r="G67" s="434" t="n">
-        <v>0.08110040354145558</v>
+        <v>0.1457</v>
       </c>
       <c r="H67" s="434" t="n">
-        <v>0.08110040354145558</v>
+        <v>0.1457</v>
       </c>
       <c r="I67" s="434" t="n">
-        <v>0.08110040354145558</v>
+        <v>0.1457</v>
       </c>
       <c r="J67" s="434" t="n">
-        <v>0.08110040354145558</v>
+        <v>0.1457</v>
       </c>
       <c r="K67" s="424" t="n">
         <v>0</v>
@@ -7025,28 +7030,28 @@
         </is>
       </c>
       <c r="C68" s="418" t="n">
-        <v>0.4191642860601364</v>
+        <v>0.4745</v>
       </c>
       <c r="D68" s="418" t="n">
-        <v>0.4116022099447514</v>
+        <v>0.5842000000000001</v>
       </c>
       <c r="E68" s="418" t="n">
-        <v>0.4403561370037248</v>
+        <v>0.4972</v>
       </c>
       <c r="F68" s="434" t="n">
-        <v>0.4237075443362042</v>
+        <v>0.4772</v>
       </c>
       <c r="G68" s="434" t="n">
-        <v>0.4137075443362042</v>
+        <v>0.4622</v>
       </c>
       <c r="H68" s="434" t="n">
-        <v>0.4037075443362042</v>
+        <v>0.4472</v>
       </c>
       <c r="I68" s="434" t="n">
-        <v>0.3937075443362042</v>
+        <v>0.4422</v>
       </c>
       <c r="J68" s="434" t="n">
-        <v>0.3837075443362042</v>
+        <v>0.4422</v>
       </c>
       <c r="K68" s="424" t="n">
         <v>-0.01</v>
@@ -7059,28 +7064,28 @@
         </is>
       </c>
       <c r="C69" s="418" t="n">
-        <v>0.1413514022209673</v>
+        <v>0.21</v>
       </c>
       <c r="D69" s="418" t="n">
-        <v>0.2433962264150944</v>
+        <v>0.21</v>
       </c>
       <c r="E69" s="418" t="n">
-        <v>0.2264547791540078</v>
+        <v>0.21</v>
       </c>
       <c r="F69" s="424" t="n">
-        <v>0.2264547791540078</v>
+        <v>0.21</v>
       </c>
       <c r="G69" s="434" t="n">
-        <v>0.2264547791540078</v>
+        <v>0.21</v>
       </c>
       <c r="H69" s="434" t="n">
-        <v>0.2264547791540078</v>
+        <v>0.21</v>
       </c>
       <c r="I69" s="434" t="n">
-        <v>0.2264547791540078</v>
+        <v>0.21</v>
       </c>
       <c r="J69" s="434" t="n">
-        <v>0.2264547791540078</v>
+        <v>0.21</v>
       </c>
       <c r="K69" s="424" t="n">
         <v>0</v>
@@ -7093,28 +7098,28 @@
         </is>
       </c>
       <c r="C70" s="418" t="n">
-        <v>0.06949429037520391</v>
+        <v>0.215</v>
       </c>
       <c r="D70" s="418" t="n">
-        <v>0.078127879122904</v>
+        <v>0.1524</v>
       </c>
       <c r="E70" s="418" t="n">
-        <v>0.08490783410138249</v>
+        <v>0.1447</v>
       </c>
       <c r="F70" s="424" t="n">
         <v>0.093</v>
       </c>
       <c r="G70" s="434" t="n">
-        <v>0.0905</v>
+        <v>0.093</v>
       </c>
       <c r="H70" s="434" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.093</v>
       </c>
       <c r="I70" s="434" t="n">
-        <v>0.08549999999999999</v>
+        <v>0.093</v>
       </c>
       <c r="J70" s="434" t="n">
-        <v>0.08299999999999999</v>
+        <v>0.093</v>
       </c>
       <c r="K70" s="424" t="n">
         <v>-0.0025</v>
@@ -8378,7 +8383,6 @@
         <v>987.5822307314286</v>
       </c>
     </row>
-    <row r="124"/>
     <row r="125">
       <c r="B125" t="inlineStr">
         <is>
@@ -8445,7 +8449,6 @@
         <v>-223</v>
       </c>
     </row>
-    <row r="128"/>
     <row r="129">
       <c r="B129" t="inlineStr">
         <is>
@@ -8987,7 +8990,6 @@
         <v>586.7181807314284</v>
       </c>
     </row>
-    <row r="154"/>
     <row r="155">
       <c r="B155" s="34" t="inlineStr">
         <is>
@@ -9126,7 +9128,6 @@
         </is>
       </c>
     </row>
-    <row r="160"/>
     <row r="161">
       <c r="B161" s="321" t="inlineStr">
         <is>
@@ -10518,7 +10519,7 @@
         </is>
       </c>
       <c r="C230" s="462" t="n">
-        <v>1660.277939999999</v>
+        <v>1203.6</v>
       </c>
       <c r="D230" s="463" t="n">
         <v>1</v>
@@ -10527,19 +10528,19 @@
         <v>1</v>
       </c>
       <c r="F230" s="417" t="n">
-        <v>5695.634218624235</v>
+        <v>3041.8</v>
       </c>
       <c r="G230" s="417" t="n">
-        <v>6309.071278125453</v>
+        <v>3220.7</v>
       </c>
       <c r="H230" s="417" t="n">
-        <v>6922.508337626672</v>
+        <v>3399.6</v>
       </c>
       <c r="I230" s="417" t="n">
-        <v>7535.945397127889</v>
+        <v>3507</v>
       </c>
       <c r="J230" s="417" t="n">
-        <v>8149.38245662911</v>
+        <v>3578.6</v>
       </c>
     </row>
     <row r="231">
@@ -11336,16 +11337,16 @@
     </row>
     <row r="260">
       <c r="B260" s="469" t="n">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="C260" s="468" t="n">
-        <v>3.430530564433228</v>
+        <v>2.377</v>
       </c>
       <c r="D260" s="166" t="n">
-        <v>0.2795941873668486</v>
+        <v>0.1891</v>
       </c>
       <c r="E260" s="417" t="n">
-        <v>-1660.277939999999</v>
+        <v>-1203.6</v>
       </c>
       <c r="F260" s="432" t="n">
         <v>0</v>
@@ -11360,21 +11361,21 @@
         <v>0</v>
       </c>
       <c r="J260" s="415" t="n">
-        <v>5695.634218624235</v>
+        <v>2861</v>
       </c>
     </row>
     <row r="261">
       <c r="B261" s="469" t="n">
-        <v>6.8</v>
+        <v>7</v>
       </c>
       <c r="C261" s="468" t="n">
-        <v>3.800009098552172</v>
+        <v>2.576</v>
       </c>
       <c r="D261" s="166" t="n">
-        <v>0.3060413503798853</v>
+        <v>0.2083</v>
       </c>
       <c r="E261" s="417" t="n">
-        <v>-1660.277939999999</v>
+        <v>-1203.6</v>
       </c>
       <c r="F261" s="417" t="n">
         <v>0</v>
@@ -11389,21 +11390,21 @@
         <v>0</v>
       </c>
       <c r="J261" s="415" t="n">
-        <v>6309.071278125453</v>
+        <v>3100.2</v>
       </c>
     </row>
     <row r="262">
       <c r="B262" s="469" t="n">
-        <v>7.3</v>
+        <v>8</v>
       </c>
       <c r="C262" s="468" t="n">
-        <v>4.169487632671115</v>
+        <v>2.973</v>
       </c>
       <c r="D262" s="166" t="n">
-        <v>0.3305050828444873</v>
+        <v>0.2435</v>
       </c>
       <c r="E262" s="417" t="n">
-        <v>-1660.277939999999</v>
+        <v>-1203.6</v>
       </c>
       <c r="F262" s="417" t="n">
         <v>0</v>
@@ -11418,21 +11419,21 @@
         <v>0</v>
       </c>
       <c r="J262" s="415" t="n">
-        <v>6922.508337626672</v>
+        <v>3578.6</v>
       </c>
     </row>
     <row r="263">
       <c r="B263" s="469" t="n">
-        <v>7.8</v>
+        <v>9</v>
       </c>
       <c r="C263" s="468" t="n">
-        <v>4.538966166790057</v>
+        <v>3.371</v>
       </c>
       <c r="D263" s="166" t="n">
-        <v>0.3532916093100265</v>
+        <v>0.2751</v>
       </c>
       <c r="E263" s="417" t="n">
-        <v>-1660.277939999999</v>
+        <v>-1203.6</v>
       </c>
       <c r="F263" s="417" t="n">
         <v>0</v>
@@ -11447,21 +11448,21 @@
         <v>0</v>
       </c>
       <c r="J263" s="415" t="n">
-        <v>7535.945397127889</v>
+        <v>4057</v>
       </c>
     </row>
     <row r="264">
       <c r="B264" s="469" t="n">
-        <v>8.300000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="C264" s="468" t="n">
-        <v>4.908444700909001</v>
+        <v>3.569</v>
       </c>
       <c r="D264" s="166" t="n">
-        <v>0.3746393777884374</v>
+        <v>0.2898</v>
       </c>
       <c r="E264" s="417" t="n">
-        <v>-1660.277939999999</v>
+        <v>-1203.6</v>
       </c>
       <c r="F264" s="417" t="n">
         <v>0</v>
@@ -11476,13 +11477,13 @@
         <v>0</v>
       </c>
       <c r="J264" s="415" t="n">
-        <v>8149.38245662911</v>
+        <v>4296.2</v>
       </c>
     </row>
     <row r="266">
       <c r="B266" s="317" t="inlineStr">
         <is>
-          <t>SUMMARY AT 7.3x EXIT EBITDA MULTIPLE</t>
+          <t>SUMMARY AT 8.0x EXIT EBITDA MULTIPLE — ZoomInfo LBOMODEL1</t>
         </is>
       </c>
       <c r="C266" s="15" t="n"/>
@@ -11679,19 +11680,19 @@
         </is>
       </c>
       <c r="F275" s="471" t="n">
-        <v>1660.277939999999</v>
+        <v>1203.6</v>
       </c>
       <c r="G275" s="472" t="n">
-        <v>0.2423567429059611</v>
+        <v>0.4185</v>
       </c>
       <c r="H275" s="472" t="n">
         <v>1</v>
       </c>
       <c r="I275" s="468" t="n">
-        <v>4.169487632671115</v>
+        <v>2.973</v>
       </c>
       <c r="J275" s="473" t="n">
-        <v>0.3305050828444873</v>
+        <v>0.2435</v>
       </c>
     </row>
     <row r="276">
@@ -12487,7 +12488,6 @@
         <v>0.2849090713511313</v>
       </c>
     </row>
-    <row r="318"/>
     <row r="319">
       <c r="B319" s="317" t="inlineStr">
         <is>
@@ -14050,7 +14050,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:K118"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="1.7109375" customWidth="1" style="244" min="1" max="1"/>
     <col width="40.28515625" customWidth="1" style="244" min="2" max="2"/>
@@ -14976,7 +14976,6 @@
         <v>0.7748616857223557</v>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
@@ -15389,7 +15388,6 @@
         <v>36.4886239211832</v>
       </c>
     </row>
-    <row r="82"/>
     <row r="83" ht="17.25" customHeight="1" s="244">
       <c r="C83" s="112" t="inlineStr">
         <is>
@@ -15565,7 +15563,6 @@
       <c r="D93" s="93" t="n"/>
       <c r="E93" s="93" t="n"/>
     </row>
-    <row r="94"/>
     <row r="114">
       <c r="B114" s="108" t="n"/>
       <c r="C114" s="109" t="inlineStr">
@@ -15683,7 +15680,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:E28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="1.7109375" customWidth="1" style="244" min="1" max="1"/>
     <col width="36.5703125" bestFit="1" customWidth="1" style="244" min="2" max="2"/>
@@ -15988,7 +15985,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A2:F268"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="19.42578125" bestFit="1" customWidth="1" style="244" min="1" max="1"/>
     <col width="9.28515625" bestFit="1" customWidth="1" style="244" min="2" max="5"/>
@@ -21291,14 +21288,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:C22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" style="244" min="2" max="2"/>
     <col width="100" customWidth="1" style="244" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="539" t="inlineStr">
         <is>
@@ -21313,7 +21309,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
@@ -21386,7 +21381,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
@@ -21429,7 +21423,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
@@ -21439,6 +21432,13 @@
       <c r="C19" t="inlineStr">
         <is>
           <t>SDR % of S&amp;M and AI unit costs are yellow assumptions. Illustrative — not investment advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>LBOMODEL1: core LBO sheet inputs now use these ZoomInfo figures (see LBO tab).</t>
         </is>
       </c>
     </row>
@@ -21457,8 +21457,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:F38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="42" customWidth="1" style="244" min="2" max="2"/>
     <col width="12" customWidth="1" style="244" min="3" max="3"/>
@@ -21467,7 +21467,6 @@
     <col width="70" customWidth="1" style="244" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="539" t="inlineStr">
         <is>
@@ -21475,7 +21474,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="541" t="inlineStr">
         <is>
@@ -21509,13 +21507,13 @@
           <t>Revenue</t>
         </is>
       </c>
-      <c r="C5" s="543" t="n">
+      <c r="C5" s="556" t="n">
         <v>1239.5</v>
       </c>
-      <c r="D5" s="543" t="n">
+      <c r="D5" s="556" t="n">
         <v>1214.3</v>
       </c>
-      <c r="E5" s="543" t="n">
+      <c r="E5" s="556" t="n">
         <v>1249.5</v>
       </c>
       <c r="F5" s="542" t="inlineStr">
@@ -21530,13 +21528,13 @@
           <t>Selling &amp; Marketing</t>
         </is>
       </c>
-      <c r="C6" s="543" t="n">
+      <c r="C6" s="556" t="n">
         <v>408.5</v>
       </c>
-      <c r="D6" s="543" t="n">
+      <c r="D6" s="556" t="n">
         <v>414.1</v>
       </c>
-      <c r="E6" s="543" t="n">
+      <c r="E6" s="556" t="n">
         <v>414.6</v>
       </c>
       <c r="F6" s="542" t="inlineStr">
@@ -21551,13 +21549,13 @@
           <t>Research &amp; Development</t>
         </is>
       </c>
-      <c r="C7" s="543" t="n">
+      <c r="C7" s="556" t="n">
         <v>191.5</v>
       </c>
-      <c r="D7" s="543" t="n">
+      <c r="D7" s="556" t="n">
         <v>196.1</v>
       </c>
-      <c r="E7" s="543" t="n">
+      <c r="E7" s="556" t="n">
         <v>182</v>
       </c>
       <c r="F7" s="542" t="inlineStr">
@@ -21572,13 +21570,13 @@
           <t>General &amp; Administrative</t>
         </is>
       </c>
-      <c r="C8" s="543" t="n">
+      <c r="C8" s="556" t="n">
         <v>179.6</v>
       </c>
-      <c r="D8" s="543" t="n">
+      <c r="D8" s="556" t="n">
         <v>295.3</v>
       </c>
-      <c r="E8" s="543" t="n">
+      <c r="E8" s="556" t="n">
         <v>206.7</v>
       </c>
       <c r="F8" s="542" t="inlineStr">
@@ -21593,7 +21591,7 @@
           <t>Operating expenses (ex-COGS)</t>
         </is>
       </c>
-      <c r="E9" s="543" t="n">
+      <c r="E9" s="556" t="n">
         <v>824.2</v>
       </c>
       <c r="F9" s="542" t="inlineStr">
@@ -21608,13 +21606,13 @@
           <t>Operating income</t>
         </is>
       </c>
-      <c r="C10" s="543" t="n">
+      <c r="C10" s="556" t="n">
         <v>259.5</v>
       </c>
-      <c r="D10" s="543" t="n">
+      <c r="D10" s="556" t="n">
         <v>97.40000000000001</v>
       </c>
-      <c r="E10" s="543" t="n">
+      <c r="E10" s="556" t="n">
         <v>225.7</v>
       </c>
       <c r="F10" s="542" t="inlineStr">
@@ -21629,13 +21627,13 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C11" s="543" t="n">
+      <c r="C11" s="556" t="n">
         <v>19.6</v>
       </c>
-      <c r="D11" s="543" t="n">
+      <c r="D11" s="556" t="n">
         <v>25.9</v>
       </c>
-      <c r="E11" s="543" t="n">
+      <c r="E11" s="556" t="n">
         <v>30.3</v>
       </c>
       <c r="F11" s="542" t="inlineStr">
@@ -21650,13 +21648,13 @@
           <t>Amort. of intangibles</t>
         </is>
       </c>
-      <c r="C12" s="543" t="n">
+      <c r="C12" s="556" t="n">
         <v>61</v>
       </c>
-      <c r="D12" s="543" t="n">
+      <c r="D12" s="556" t="n">
         <v>59.8</v>
       </c>
-      <c r="E12" s="543" t="n">
+      <c r="E12" s="556" t="n">
         <v>58.5</v>
       </c>
       <c r="F12" s="542" t="inlineStr">
@@ -21671,13 +21669,13 @@
           <t>Total D&amp;A (dep+intang)</t>
         </is>
       </c>
-      <c r="C13" s="543" t="n">
+      <c r="C13" s="556" t="n">
         <v>80.59999999999999</v>
       </c>
-      <c r="D13" s="543" t="n">
+      <c r="D13" s="556" t="n">
         <v>85.7</v>
       </c>
-      <c r="E13" s="543" t="n">
+      <c r="E13" s="556" t="n">
         <v>88.8</v>
       </c>
       <c r="F13" s="542" t="inlineStr">
@@ -21692,13 +21690,13 @@
           <t>Share-based compensation</t>
         </is>
       </c>
-      <c r="C14" s="543" t="n">
+      <c r="C14" s="556" t="n">
         <v>167.6</v>
       </c>
-      <c r="D14" s="543" t="n">
+      <c r="D14" s="556" t="n">
         <v>138</v>
       </c>
-      <c r="E14" s="543" t="n">
+      <c r="E14" s="556" t="n">
         <v>116.2</v>
       </c>
       <c r="F14" s="542" t="inlineStr">
@@ -21713,7 +21711,7 @@
           <t>Advertising expense</t>
         </is>
       </c>
-      <c r="E15" s="543" t="n">
+      <c r="E15" s="556" t="n">
         <v>37.3</v>
       </c>
       <c r="F15" s="542" t="inlineStr">
@@ -21728,13 +21726,13 @@
           <t>Amort. deferred commissions</t>
         </is>
       </c>
-      <c r="C16" s="543" t="n">
+      <c r="C16" s="556" t="n">
         <v>75.3</v>
       </c>
-      <c r="D16" s="543" t="n">
+      <c r="D16" s="556" t="n">
         <v>67.59999999999999</v>
       </c>
-      <c r="E16" s="543" t="n">
+      <c r="E16" s="556" t="n">
         <v>90.2</v>
       </c>
       <c r="F16" s="542" t="inlineStr">
@@ -21749,13 +21747,13 @@
           <t>Net income</t>
         </is>
       </c>
-      <c r="C17" s="543" t="n">
+      <c r="C17" s="556" t="n">
         <v>107.3</v>
       </c>
-      <c r="D17" s="543" t="n">
+      <c r="D17" s="556" t="n">
         <v>29.1</v>
       </c>
-      <c r="E17" s="543" t="n">
+      <c r="E17" s="556" t="n">
         <v>124.2</v>
       </c>
       <c r="F17" s="542" t="inlineStr">
@@ -21764,14 +21762,13 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="544" t="inlineStr">
         <is>
           <t>Implied COGS (Rev − OpEx − OpInc)</t>
         </is>
       </c>
-      <c r="E19" s="545">
+      <c r="E19" s="557">
         <f>E5-E9-E10</f>
         <v/>
       </c>
@@ -21782,7 +21779,7 @@
           <t>GAAP EBITDA proxy (OpInc + D&amp;A)</t>
         </is>
       </c>
-      <c r="E20" s="545">
+      <c r="E20" s="557">
         <f>E10+E13</f>
         <v/>
       </c>
@@ -21804,7 +21801,7 @@
           <t>Adj. EBITDA proxy (+SBC)</t>
         </is>
       </c>
-      <c r="E22" s="545">
+      <c r="E22" s="557">
         <f>E20+E14</f>
         <v/>
       </c>
@@ -21820,7 +21817,6 @@
         <v/>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="B25" s="547" t="inlineStr">
         <is>
@@ -21895,7 +21891,7 @@
           <t>S&amp;M $ / S&amp;M employee ($000s)</t>
         </is>
       </c>
-      <c r="E32" s="545">
+      <c r="E32" s="557">
         <f>E6*1000/E28</f>
         <v/>
       </c>
@@ -21911,7 +21907,6 @@
         <v/>
       </c>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="B35" s="542" t="inlineStr">
         <is>
@@ -21942,14 +21937,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:C21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="48" customWidth="1" style="244" min="2" max="2"/>
     <col width="14" customWidth="1" style="244" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="539" t="inlineStr">
         <is>
@@ -21957,14 +21951,13 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="542" t="inlineStr">
         <is>
           <t>FY2025 Revenue ($m)</t>
         </is>
       </c>
-      <c r="C4" s="545">
+      <c r="C4" s="557">
         <f>'ZI_01_10K_Source'!E5</f>
         <v/>
       </c>
@@ -21975,7 +21968,7 @@
           <t>FY2025 S&amp;M ($m)</t>
         </is>
       </c>
-      <c r="C5" s="545">
+      <c r="C5" s="557">
         <f>'ZI_01_10K_Source'!E6</f>
         <v/>
       </c>
@@ -21991,7 +21984,6 @@
         <v/>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="B8" s="547" t="inlineStr">
         <is>
@@ -22005,7 +21997,7 @@
           <t>Advertising</t>
         </is>
       </c>
-      <c r="C9" s="545">
+      <c r="C9" s="557">
         <f>'ZI_01_10K_Source'!E15</f>
         <v/>
       </c>
@@ -22016,7 +22008,7 @@
           <t>Deferred commission amortization</t>
         </is>
       </c>
-      <c r="C10" s="545">
+      <c r="C10" s="557">
         <f>'ZI_01_10K_Source'!E16</f>
         <v/>
       </c>
@@ -22027,7 +22019,7 @@
           <t>Residual S&amp;M (people + other)</t>
         </is>
       </c>
-      <c r="C11" s="545">
+      <c r="C11" s="557">
         <f>C5-C9-C10</f>
         <v/>
       </c>
@@ -22049,12 +22041,11 @@
           <t>Residual $ / S&amp;M employee ($000s)</t>
         </is>
       </c>
-      <c r="C13" s="545">
+      <c r="C13" s="557">
         <f>C11*1000/'ZI_01_10K_Source'!E28</f>
         <v/>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="B15" s="547" t="inlineStr">
         <is>
@@ -22078,7 +22069,7 @@
           <t>S&amp;M bloat vs target ($m)</t>
         </is>
       </c>
-      <c r="C17" s="545">
+      <c r="C17" s="557">
         <f>MAX(0,C5-C4*C16)</f>
         <v/>
       </c>
@@ -22105,7 +22096,6 @@
         <v/>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
@@ -22124,8 +22114,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:E40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="48" customWidth="1" style="244" min="2" max="2"/>
     <col width="12" customWidth="1" style="244" min="3" max="3"/>
@@ -22133,7 +22123,6 @@
     <col width="12" customWidth="1" style="244" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="539" t="inlineStr">
         <is>
@@ -22141,7 +22130,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="547" t="inlineStr">
         <is>
@@ -22187,7 +22175,7 @@
           <t>Fully loaded cost / SDR / yr ($000s)</t>
         </is>
       </c>
-      <c r="C8" s="543" t="n">
+      <c r="C8" s="556" t="n">
         <v>155</v>
       </c>
     </row>
@@ -22197,12 +22185,11 @@
           <t>Addressable SDR cost pool ($m)</t>
         </is>
       </c>
-      <c r="C9" s="545">
+      <c r="C9" s="557">
         <f>C7*C8/1000</f>
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="B11" s="547" t="inlineStr">
         <is>
@@ -22226,7 +22213,7 @@
           <t>AI platform + compute / seat / yr ($000s)</t>
         </is>
       </c>
-      <c r="C13" s="543" t="n">
+      <c r="C13" s="556" t="n">
         <v>15</v>
       </c>
     </row>
@@ -22246,7 +22233,7 @@
           <t>Oversight fully loaded / FTE / yr ($000s)</t>
         </is>
       </c>
-      <c r="C15" s="543" t="n">
+      <c r="C15" s="556" t="n">
         <v>150</v>
       </c>
     </row>
@@ -22256,7 +22243,7 @@
           <t>One-time severance / SDR ($000s)</t>
         </is>
       </c>
-      <c r="C16" s="543" t="n">
+      <c r="C16" s="556" t="n">
         <v>25</v>
       </c>
     </row>
@@ -22266,11 +22253,10 @@
           <t>One-time AI build / integration ($m) in Y1</t>
         </is>
       </c>
-      <c r="C17" s="543" t="n">
+      <c r="C17" s="556" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="547" t="inlineStr">
         <is>
@@ -22373,20 +22359,19 @@
           <t>Avg SDRs during year</t>
         </is>
       </c>
-      <c r="C25" s="545">
+      <c r="C25" s="557">
         <f>($C$7+C22)/2</f>
         <v/>
       </c>
-      <c r="D25" s="545">
+      <c r="D25" s="557">
         <f>(C22+D22)/2</f>
         <v/>
       </c>
-      <c r="E25" s="545">
+      <c r="E25" s="557">
         <f>(D22+E22)/2</f>
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="B27" s="547" t="inlineStr">
         <is>
@@ -22400,15 +22385,15 @@
           <t>AI seats (cum.)</t>
         </is>
       </c>
-      <c r="C28" s="545">
+      <c r="C28" s="557">
         <f>C23*$C$12</f>
         <v/>
       </c>
-      <c r="D28" s="545">
+      <c r="D28" s="557">
         <f>D23*$C$12</f>
         <v/>
       </c>
-      <c r="E28" s="545">
+      <c r="E28" s="557">
         <f>E23*$C$12</f>
         <v/>
       </c>
@@ -22432,7 +22417,6 @@
         <v/>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="B31" s="547" t="inlineStr">
         <is>
@@ -22446,15 +22430,15 @@
           <t>SDR cash cost (avg HC × cost)</t>
         </is>
       </c>
-      <c r="C32" s="545">
+      <c r="C32" s="557">
         <f>C25*$C$8/1000</f>
         <v/>
       </c>
-      <c r="D32" s="545">
+      <c r="D32" s="557">
         <f>D25*$C$8/1000</f>
         <v/>
       </c>
-      <c r="E32" s="545">
+      <c r="E32" s="557">
         <f>E25*$C$8/1000</f>
         <v/>
       </c>
@@ -22465,15 +22449,15 @@
           <t>Baseline SDR cost if no program</t>
         </is>
       </c>
-      <c r="C33" s="545">
+      <c r="C33" s="557">
         <f>$C$9</f>
         <v/>
       </c>
-      <c r="D33" s="545">
+      <c r="D33" s="557">
         <f>$C$9</f>
         <v/>
       </c>
-      <c r="E33" s="545">
+      <c r="E33" s="557">
         <f>$C$9</f>
         <v/>
       </c>
@@ -22484,15 +22468,15 @@
           <t>Gross SDR savings vs baseline</t>
         </is>
       </c>
-      <c r="C34" s="545">
+      <c r="C34" s="557">
         <f>C33-C32</f>
         <v/>
       </c>
-      <c r="D34" s="545">
+      <c r="D34" s="557">
         <f>D33-D32</f>
         <v/>
       </c>
-      <c r="E34" s="545">
+      <c r="E34" s="557">
         <f>E33-E32</f>
         <v/>
       </c>
@@ -22503,15 +22487,15 @@
           <t>AI seat opex</t>
         </is>
       </c>
-      <c r="C35" s="545">
+      <c r="C35" s="557">
         <f>C28*$C$13/1000</f>
         <v/>
       </c>
-      <c r="D35" s="545">
+      <c r="D35" s="557">
         <f>D28*$C$13/1000</f>
         <v/>
       </c>
-      <c r="E35" s="545">
+      <c r="E35" s="557">
         <f>E28*$C$13/1000</f>
         <v/>
       </c>
@@ -22522,15 +22506,15 @@
           <t>Oversight opex</t>
         </is>
       </c>
-      <c r="C36" s="545">
+      <c r="C36" s="557">
         <f>C29*$C$15/1000</f>
         <v/>
       </c>
-      <c r="D36" s="545">
+      <c r="D36" s="557">
         <f>D29*$C$15/1000</f>
         <v/>
       </c>
-      <c r="E36" s="545">
+      <c r="E36" s="557">
         <f>E29*$C$15/1000</f>
         <v/>
       </c>
@@ -22541,15 +22525,15 @@
           <t>Severance (this year's exits)</t>
         </is>
       </c>
-      <c r="C37" s="545">
+      <c r="C37" s="557">
         <f>C24*$C$16/1000</f>
         <v/>
       </c>
-      <c r="D37" s="545">
+      <c r="D37" s="557">
         <f>D24*$C$16/1000</f>
         <v/>
       </c>
-      <c r="E37" s="545">
+      <c r="E37" s="557">
         <f>E24*$C$16/1000</f>
         <v/>
       </c>
@@ -22560,14 +22544,14 @@
           <t>AI build (Y1 only)</t>
         </is>
       </c>
-      <c r="C38" s="545">
+      <c r="C38" s="557">
         <f>$C$17</f>
         <v/>
       </c>
-      <c r="D38" s="543" t="n">
-        <v>0</v>
-      </c>
-      <c r="E38" s="543" t="n">
+      <c r="D38" s="556" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="556" t="n">
         <v>0</v>
       </c>
     </row>
@@ -22577,15 +22561,15 @@
           <t>Net EBITDA benefit (in-year, after one-time)</t>
         </is>
       </c>
-      <c r="C39" s="545">
+      <c r="C39" s="557">
         <f>C34-C35-C36-C37-C38</f>
         <v/>
       </c>
-      <c r="D39" s="545">
+      <c r="D39" s="557">
         <f>D34-D35-D36-D37-D38</f>
         <v/>
       </c>
-      <c r="E39" s="545">
+      <c r="E39" s="557">
         <f>E34-E35-E36-E37-E38</f>
         <v/>
       </c>
@@ -22596,15 +22580,15 @@
           <t>Year-end run-rate benefit (ex one-time)</t>
         </is>
       </c>
-      <c r="C40" s="545">
+      <c r="C40" s="557">
         <f>(C23*$C$8/1000)-(C28*$C$13/1000)-(C29*$C$15/1000)</f>
         <v/>
       </c>
-      <c r="D40" s="545">
+      <c r="D40" s="557">
         <f>(D23*$C$8/1000)-(D28*$C$13/1000)-(D29*$C$15/1000)</f>
         <v/>
       </c>
-      <c r="E40" s="545">
+      <c r="E40" s="557">
         <f>(E23*$C$8/1000)-(E28*$C$13/1000)-(E29*$C$15/1000)</f>
         <v/>
       </c>

</xml_diff>